<commit_message>
S136 4절: 마감 - 1번 PC 1,681건 3분 58초 · 회귀 118/118 · 미해결 67 -> 64
지시서를 docs\directives\S136.md 에 앉혔다 (제어문자 0 · 탭 0).
앞단 전체 pytest 두 판 - 고치기 전 3분 58초(깨끗한 판, 표에 넣은 값) ·
고친 뒤 3분 40초(앞을 안 봤고 뒤에 site-energy python 둘 - 견주지 않는다).
둘 다 1,680 passed · 1 xfailed · failed 0 · skip 0 · 수집 1,681건.
케이스 118/118 · 회귀값 여덟 불변 · 화면 감사 넷 불변(957 807 961 808) ·
규칙 위반 없음. 덱 small-b-sell 에서 MWh 두 꼴이 그대로인 것을 글자로 봤다
(3장 표 984.2 MWh · 4장 지표 984 MWh).
살아 있는 못 1 -> 1.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>12.09962279999991</v>
+        <v>12.5498047000001</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>10.67046060000007</v>
+        <v>12.36363039999969</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>7.862946800000032</v>
+        <v>7.696366500000295</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>12.26684360000002</v>
+        <v>12.24796730000025</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>12.12214440000002</v>
+        <v>14.17616560000033</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>9.679036499999938</v>
+        <v>9.36924689999978</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>13.07896449999998</v>
+        <v>11.38146289999986</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>15.77080739999997</v>
+        <v>16.60361299999977</v>
       </c>
     </row>
   </sheetData>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12.1 초</t>
+          <t>12.5 초</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10.7 초</t>
+          <t>12.4 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7.9 초</t>
+          <t>7.7 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12.3 초</t>
+          <t>12.2 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.1 초</t>
+          <t>14.2 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>9.7 초</t>
+          <t>9.4 초</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.1 초</t>
+          <t>11.4 초</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.8 초</t>
+          <t>16.6 초</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>98.6 초</t>
+          <t>100.0 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S138 4절: 마감 - 1,682건 3분 39초 · 케이스 118/118 · 감사 넷 불변 (미해결 67 -> 69)
Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>11.55603249999967</v>
+        <v>9.862520299999233</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>10.74174920000041</v>
+        <v>9.805634899999859</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>7.808038199999828</v>
+        <v>6.767232999998669</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>12.63888080000015</v>
+        <v>10.15034410000044</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>12.24405750000005</v>
+        <v>10.77493789999971</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>10.85559840000042</v>
+        <v>8.8462974999984</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>12.32665139999972</v>
+        <v>10.34146320000036</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>17.14594020000004</v>
+        <v>14.31703560000096</v>
       </c>
     </row>
   </sheetData>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11.6 초</t>
+          <t>9.9 초</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10.7 초</t>
+          <t>9.8 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7.8 초</t>
+          <t>6.8 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>12.6 초</t>
+          <t>10.2 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>12.2 초</t>
+          <t>10.8 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.9 초</t>
+          <t>8.8 초</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>12.3 초</t>
+          <t>10.3 초</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>17.1 초</t>
+          <t>14.3 초</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>98.9 초</t>
+          <t>84.1 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S139 4절: 마감 - 1,682건 3분 46초 · 케이스 118/118 · 감사 넷 불변 (미해결 69 -> 69)
pytest 1,681 passed · 1 xfailed · failed 0 · skip 0 (수집 1,682건 · 1번 PC ·
앞단 전체 · 깨끗한 판). 건수가 앞 판과 같다 - 시험을 더하지 않았다.
케이스 118/118 · 회귀값 여덟 불변 · 기상 취득 0회 (도구 100.8초 / 벽시계 105초).
화면 감사 넷 불변 (957 · 807 · 961 · 808).
ruff check 통과 · ruff format 어긋남 여덟 · mypy 10건 (둘 다 앞 판과 같다).

미해결 69 -> 69. 늘어난 것 하나 - 「PPT 용어집이 요금적용전력을 「기본요금을
매기는 전력」 이라 적는다」. 줄어든 것 하나 - 「부록 계산 근거의 기본요금 산식이
제 값을 안 낸다」.

3절은 건너뛰었다 - 1번 PC 라 2번 PC 의 「무엇이 먹나」 를 못 잰다.
살아 있는 못 1건 (test_excess.py 의 xfail strict) - 앞 판과 같다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>9.862520299999233</v>
+        <v>12.22277810000014</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>9.805634899999859</v>
+        <v>10.77358199999981</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>6.767232999998669</v>
+        <v>7.747335100000782</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>10.15034410000044</v>
+        <v>12.99014390000048</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>10.77493789999971</v>
+        <v>12.18056849999994</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>8.8462974999984</v>
+        <v>10.58264869999948</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>10.34146320000036</v>
+        <v>12.11081969999941</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>14.31703560000096</v>
+        <v>18.80785629999991</v>
       </c>
     </row>
   </sheetData>
@@ -10469,7 +10469,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9.9 초</t>
+          <t>12.2 초</t>
         </is>
       </c>
     </row>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9.8 초</t>
+          <t>10.8 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6.8 초</t>
+          <t>7.7 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.2 초</t>
+          <t>13.0 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10.8 초</t>
+          <t>12.2 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>8.8 초</t>
+          <t>10.6 초</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10.3 초</t>
+          <t>12.1 초</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.3 초</t>
+          <t>18.8 초</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>84.1 초</t>
+          <t>100.8 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S141 5절: 마감 - 1,685건 3분 25초 · 케이스 118/118 · 감사 넷 불변 (미해결 71 -> 68)
pytest 1,685 passed · xfailed 0 · failed 0 · skip 0 (수집 1,685건 · 1번 PC ·
앞단 전체 · 일꾼 8 · 깨끗한 판). 건수가 1,683 -> 1,685 로 둘 늘었다 —
tests\test_base_fee_definition.py 가 정의 못 둘을 세웠다. 앞 판에
test_doc_counts 1건이 빨갰다 — 새 파일이 1 엔진 갈래에 들어 문서의 파일 수가
낡았고 26 -> 27 로 고쳤다.

케이스 118/118 · 회귀값 여덟 불변 · 도구 84.3초 / 벽시계 89초 · 기상 취득 0회.
화면 감사 957·807·961·808 불변. scan_ctrl 제어문자 0 · 탭 0.
ruff check 통과 · ruff format 어긋남 여덟(기존) · mypy 10건(기존).
살아 있는 못 0건.

미해결 71 -> 68. 줄어든 것 셋 — capture_screen 의 드롭다운 대기가 고정 시간이라
기계가 바쁘면 깨진다 · capture_screen 이 기계가 놀 때도 전압구분에서 죽는다 ·
「기본요금」 이 산출물마다 다른 몫을 센다. 늘어난 것 없음.

4절(2번 PC 「무엇이 먹나」)은 1번 PC 라 건너뛰었다.
백그라운드 셸 없다 — 앞단으로만 돌렸고 마감에 남의 python 0개를 봤다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>9.693287100000816</v>
+        <v>9.723912499997823</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>9.698256499999843</v>
+        <v>9.773525199998403</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>6.44897999999921</v>
+        <v>6.62084859999959</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>9.853801899998871</v>
+        <v>10.140537700001</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>10.60158720000072</v>
+        <v>10.88950670000122</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>8.271002499999668</v>
+        <v>8.517785000000003</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>9.97084360000008</v>
+        <v>10.14133120000042</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>14.06810589999986</v>
+        <v>15.18163450000065</v>
       </c>
     </row>
   </sheetData>
@@ -10481,7 +10481,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9.7 초</t>
+          <t>9.8 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +10493,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6.4 초</t>
+          <t>6.6 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +10505,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>9.9 초</t>
+          <t>10.1 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +10517,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10.6 초</t>
+          <t>10.9 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +10529,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>8.3 초</t>
+          <t>8.5 초</t>
         </is>
       </c>
     </row>
@@ -10541,7 +10541,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10.0 초</t>
+          <t>10.1 초</t>
         </is>
       </c>
     </row>
@@ -10553,7 +10553,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.1 초</t>
+          <t>15.2 초</t>
         </is>
       </c>
     </row>
@@ -10565,7 +10565,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>81.8 초</t>
+          <t>84.3 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S142 5절: 마감 - 1,688건 3분 30초 · 케이스 132/132 · 감사 넷 불변 (미해결 68 -> 67)
pytest 1,688 passed · xfailed 0 · failed 0 · skip 0 (수집 1,688건 · 1번 PC ·
앞단 전체 · 깨끗한 판). 건수가 셋 는 것은 이 판이 세운 못 셋이다.

케이스 132/132 · 도구 103.6초 / 벽시계 108초 · 기상 취득 0회 · 회귀값 여덟
불변. 케이스가 여덟에서 아홉이 됐다 — C8 이 붙어 판정 118 -> 132 다.

감사 넷 불변 (957·807·961·808) · scan_ctrl 0곳 · ruff check 통과 ·
ruff format 8파일(앞 판과 같다) · mypy 통과 · 살아 있는 못 0건.

세션 목록표에 141세션 행이 빠져 있어 채웠다 — 그 판이 절만 남기고 표에
행을 안 남겼다. 지어내지 않고 그 절에서 옮겼다.

mypy 는 「기존 10건」 이 아니다 — 실물은 no issues found in 110 source files
다. 고치지 않고 사실만 적는다.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -420,7 +420,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>9.723912499997823</v>
+        <v>10.29694350000136</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>9.773525199998403</v>
+        <v>10.41423510000095</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>6.62084859999959</v>
+        <v>7.360852599998907</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>10.140537700001</v>
+        <v>11.33471169999757</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>10.88950670000122</v>
+        <v>11.83807510000042</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>8.517785000000003</v>
+        <v>9.069716400001198</v>
       </c>
     </row>
     <row r="8">
@@ -856,59 +856,111 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>10.14133120000042</v>
+        <v>10.55809339999905</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>C8 역률 미달형</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>general_b</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>2023-04-25 ~ 2024-04-27</t>
+        </is>
+      </c>
+      <c r="D9" t="n">
+        <v>22284.79992</v>
+      </c>
+      <c r="E9" t="n">
+        <v>5293.44</v>
+      </c>
+      <c r="F9" t="n">
+        <v>5293</v>
+      </c>
+      <c r="G9" t="n">
+        <v>49.01480732181292</v>
+      </c>
+      <c r="H9" t="n">
+        <v>64.95604774948416</v>
+      </c>
+      <c r="I9" t="n">
+        <v>459143820.0375</v>
+      </c>
+      <c r="J9" t="n">
+        <v>2898284725.008</v>
+      </c>
+      <c r="K9" t="n">
+        <v>3357428545.0455</v>
+      </c>
+      <c r="L9" t="n">
+        <v>13.67546066512869</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>cache</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>12.74110610000207</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>R1 용인 실측</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="B10" t="inlineStr">
         <is>
           <t>general_a_2</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>2025-08-28 ~ 2026-08-28</t>
         </is>
       </c>
-      <c r="D9" t="n">
+      <c r="D10" t="n">
         <v>476.02327</v>
       </c>
-      <c r="E9" t="n">
+      <c r="E10" t="n">
         <v>132.28</v>
       </c>
-      <c r="F9" t="n">
+      <c r="F10" t="n">
         <v>132</v>
       </c>
-      <c r="G9" t="n">
+      <c r="G10" t="n">
         <v>41.08229342532648</v>
       </c>
-      <c r="H9" t="n">
+      <c r="H10" t="n">
         <v>100.8144862191238</v>
       </c>
-      <c r="I9" t="n">
+      <c r="I10" t="n">
         <v>12422521.29032258</v>
       </c>
-      <c r="J9" t="n">
+      <c r="J10" t="n">
         <v>49597412.23</v>
       </c>
-      <c r="K9" t="n">
+      <c r="K10" t="n">
         <v>62019933.52032258</v>
       </c>
-      <c r="L9" t="n">
+      <c r="L10" t="n">
         <v>20.02988488572306</v>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>cache</t>
         </is>
       </c>
-      <c r="N9" t="n">
-        <v>15.18163450000065</v>
+      <c r="N10" t="n">
+        <v>16.1661595000005</v>
       </c>
     </row>
   </sheetData>
@@ -922,7 +974,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L33"/>
+  <dimension ref="A1:L37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1879,7 +1931,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C8 역률 미달형</t>
         </is>
       </c>
       <c r="B30" t="n">
@@ -1893,7 +1945,7 @@
         <v>0</v>
       </c>
       <c r="F30" t="n">
-        <v>132</v>
+        <v>5293</v>
       </c>
       <c r="G30" t="n">
         <v>0</v>
@@ -1915,28 +1967,28 @@
         <v>500</v>
       </c>
       <c r="C31" t="n">
-        <v>653924.9987308802</v>
+        <v>584346.8725203483</v>
       </c>
       <c r="D31" t="n">
-        <v>28.80135248983531</v>
+        <v>100</v>
       </c>
       <c r="E31" t="n">
-        <v>465585.7548272483</v>
+        <v>0</v>
       </c>
       <c r="F31" t="n">
-        <v>120</v>
+        <v>5204</v>
       </c>
       <c r="G31" t="n">
-        <v>1371755.161290321</v>
+        <v>12693662.5</v>
       </c>
       <c r="H31" t="n">
-        <v>21832794.0374309</v>
+        <v>78883246.71788597</v>
       </c>
       <c r="I31" t="n">
-        <v>23204549.19872123</v>
+        <v>91754620.49288607</v>
       </c>
       <c r="J31" t="n">
-        <v>23204549.19872123</v>
+        <v>91754620.49288607</v>
       </c>
       <c r="K31" t="inlineStr"/>
       <c r="L31" t="inlineStr"/>
@@ -1946,28 +1998,28 @@
         <v>1000</v>
       </c>
       <c r="C32" t="n">
-        <v>1307849.99746176</v>
+        <v>1168693.745040697</v>
       </c>
       <c r="D32" t="n">
-        <v>15.68075433387349</v>
+        <v>100</v>
       </c>
       <c r="E32" t="n">
-        <v>1102769.252304211</v>
+        <v>0</v>
       </c>
       <c r="F32" t="n">
-        <v>120</v>
+        <v>5198</v>
       </c>
       <c r="G32" t="n">
-        <v>1421135.161290321</v>
+        <v>17911015</v>
       </c>
       <c r="H32" t="n">
-        <v>23715557.01062761</v>
+        <v>157766493.4357724</v>
       </c>
       <c r="I32" t="n">
-        <v>25136692.17191793</v>
+        <v>175928262.6457725</v>
       </c>
       <c r="J32" t="n">
-        <v>25136692.17191793</v>
+        <v>175928262.6457725</v>
       </c>
       <c r="K32" t="inlineStr"/>
       <c r="L32" t="inlineStr"/>
@@ -1977,37 +2029,165 @@
         <v>2000</v>
       </c>
       <c r="C33" t="n">
-        <v>2615699.994923521</v>
+        <v>2337387.490081393</v>
       </c>
       <c r="D33" t="n">
-        <v>8.179882063646165</v>
+        <v>100</v>
       </c>
       <c r="E33" t="n">
-        <v>2401738.820199978</v>
+        <v>0</v>
       </c>
       <c r="F33" t="n">
-        <v>120</v>
+        <v>5186</v>
       </c>
       <c r="G33" t="n">
-        <v>1421135.161290321</v>
+        <v>21835085</v>
       </c>
       <c r="H33" t="n">
-        <v>24660958.77724204</v>
+        <v>315532986.8715444</v>
       </c>
       <c r="I33" t="n">
-        <v>26082093.93853237</v>
+        <v>337673763.0615444</v>
       </c>
       <c r="J33" t="n">
-        <v>26082093.93853237</v>
+        <v>337673763.0615444</v>
       </c>
       <c r="K33" t="inlineStr"/>
       <c r="L33" t="inlineStr"/>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>0</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>0</v>
+      </c>
+      <c r="F34" t="n">
+        <v>132</v>
+      </c>
+      <c r="G34" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
+      <c r="I34" t="n">
+        <v>0</v>
+      </c>
+      <c r="J34" t="n">
+        <v>0</v>
+      </c>
+      <c r="K34" t="inlineStr"/>
+      <c r="L34" t="inlineStr"/>
+    </row>
+    <row r="35">
+      <c r="B35" t="n">
+        <v>500</v>
+      </c>
+      <c r="C35" t="n">
+        <v>653924.9987308802</v>
+      </c>
+      <c r="D35" t="n">
+        <v>28.80135248983531</v>
+      </c>
+      <c r="E35" t="n">
+        <v>465585.7548272483</v>
+      </c>
+      <c r="F35" t="n">
+        <v>120</v>
+      </c>
+      <c r="G35" t="n">
+        <v>1371755.161290321</v>
+      </c>
+      <c r="H35" t="n">
+        <v>21832794.0374309</v>
+      </c>
+      <c r="I35" t="n">
+        <v>23204549.19872123</v>
+      </c>
+      <c r="J35" t="n">
+        <v>23204549.19872123</v>
+      </c>
+      <c r="K35" t="inlineStr"/>
+      <c r="L35" t="inlineStr"/>
+    </row>
+    <row r="36">
+      <c r="B36" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C36" t="n">
+        <v>1307849.99746176</v>
+      </c>
+      <c r="D36" t="n">
+        <v>15.68075433387349</v>
+      </c>
+      <c r="E36" t="n">
+        <v>1102769.252304211</v>
+      </c>
+      <c r="F36" t="n">
+        <v>120</v>
+      </c>
+      <c r="G36" t="n">
+        <v>1421135.161290321</v>
+      </c>
+      <c r="H36" t="n">
+        <v>23715557.01062761</v>
+      </c>
+      <c r="I36" t="n">
+        <v>25136692.17191793</v>
+      </c>
+      <c r="J36" t="n">
+        <v>25136692.17191793</v>
+      </c>
+      <c r="K36" t="inlineStr"/>
+      <c r="L36" t="inlineStr"/>
+    </row>
+    <row r="37">
+      <c r="B37" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C37" t="n">
+        <v>2615699.994923521</v>
+      </c>
+      <c r="D37" t="n">
+        <v>8.179882063646165</v>
+      </c>
+      <c r="E37" t="n">
+        <v>2401738.820199978</v>
+      </c>
+      <c r="F37" t="n">
+        <v>120</v>
+      </c>
+      <c r="G37" t="n">
+        <v>1421135.161290321</v>
+      </c>
+      <c r="H37" t="n">
+        <v>24660958.77724204</v>
+      </c>
+      <c r="I37" t="n">
+        <v>26082093.93853237</v>
+      </c>
+      <c r="J37" t="n">
+        <v>26082093.93853237</v>
+      </c>
+      <c r="K37" t="inlineStr"/>
+      <c r="L37" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A18:A21"/>
     <mergeCell ref="A26:A29"/>
     <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A34:A37"/>
     <mergeCell ref="A6:A9"/>
     <mergeCell ref="A14:A17"/>
     <mergeCell ref="A30:A33"/>
@@ -2024,7 +2204,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I169"/>
+  <dimension ref="A1:I190"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -6270,7 +6450,7 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C8 역률 미달형</t>
         </is>
       </c>
       <c r="B149" t="n">
@@ -6282,13 +6462,13 @@
         </is>
       </c>
       <c r="D149" t="n">
-        <v>1371755.161290321</v>
+        <v>-54359243.75</v>
       </c>
       <c r="E149" t="n">
-        <v>1019989.032258064</v>
+        <v>-56468883.75</v>
       </c>
       <c r="F149" t="n">
-        <v>1421135.161290321</v>
+        <v>-54359243.75</v>
       </c>
       <c r="G149" t="inlineStr">
         <is>
@@ -6297,11 +6477,11 @@
       </c>
       <c r="H149" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I149" t="n">
-        <v>28.22716233887541</v>
+        <v>3.735933597235309</v>
       </c>
     </row>
     <row r="150">
@@ -6311,13 +6491,13 @@
         </is>
       </c>
       <c r="D150" t="n">
-        <v>21832794.0374309</v>
+        <v>198235738.4790244</v>
       </c>
       <c r="E150" t="n">
-        <v>19707849.27224809</v>
+        <v>197954047.4566307</v>
       </c>
       <c r="F150" t="n">
-        <v>23383003.92461409</v>
+        <v>198235738.4790244</v>
       </c>
       <c r="G150" t="inlineStr">
         <is>
@@ -6326,11 +6506,11 @@
       </c>
       <c r="H150" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I150" t="n">
-        <v>15.71720495884344</v>
+        <v>0.1420990102768526</v>
       </c>
     </row>
     <row r="151">
@@ -6340,13 +6520,13 @@
         </is>
       </c>
       <c r="D151" t="n">
-        <v>22552939.7162026</v>
+        <v>142168620.405767</v>
       </c>
       <c r="E151" t="n">
-        <v>20181372.38521974</v>
+        <v>139736187.0250936</v>
       </c>
       <c r="F151" t="n">
-        <v>24100050.37364634</v>
+        <v>142168620.405767</v>
       </c>
       <c r="G151" t="inlineStr">
         <is>
@@ -6355,11 +6535,11 @@
       </c>
       <c r="H151" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I151" t="n">
-        <v>16.26004065415448</v>
+        <v>1.710949556752355</v>
       </c>
     </row>
     <row r="152">
@@ -6369,13 +6549,13 @@
         </is>
       </c>
       <c r="D152" t="n">
-        <v>22552939.7162026</v>
+        <v>142168620.405767</v>
       </c>
       <c r="E152" t="n">
-        <v>20181372.38521974</v>
+        <v>139736187.0250936</v>
       </c>
       <c r="F152" t="n">
-        <v>24100050.37364634</v>
+        <v>142168620.405767</v>
       </c>
       <c r="G152" t="inlineStr">
         <is>
@@ -6384,11 +6564,11 @@
       </c>
       <c r="H152" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I152" t="n">
-        <v>16.26004065415447</v>
+        <v>1.710949556752355</v>
       </c>
     </row>
     <row r="153">
@@ -6398,13 +6578,13 @@
         </is>
       </c>
       <c r="D153" t="n">
-        <v>120</v>
+        <v>5204</v>
       </c>
       <c r="E153" t="n">
-        <v>120</v>
+        <v>5201</v>
       </c>
       <c r="F153" t="n">
-        <v>122</v>
+        <v>5209</v>
       </c>
       <c r="G153" t="inlineStr">
         <is>
@@ -6417,7 +6597,7 @@
         </is>
       </c>
       <c r="I153" t="n">
-        <v>1.639344262295082</v>
+        <v>0.1535803417162603</v>
       </c>
     </row>
     <row r="154">
@@ -6427,26 +6607,26 @@
         </is>
       </c>
       <c r="D154" t="n">
-        <v>653924.9987308802</v>
+        <v>584346.8725203483</v>
       </c>
       <c r="E154" t="n">
-        <v>653917.3979531642</v>
+        <v>584298.3051197322</v>
       </c>
       <c r="F154" t="n">
-        <v>653931.4335780952</v>
+        <v>584399.679278902</v>
       </c>
       <c r="G154" t="inlineStr">
         <is>
-          <t>첨예형</t>
+          <t>평탄형</t>
         </is>
       </c>
       <c r="H154" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>첨예형</t>
         </is>
       </c>
       <c r="I154" t="n">
-        <v>0.002146345046327881</v>
+        <v>0.01734671711232556</v>
       </c>
     </row>
     <row r="155">
@@ -6480,13 +6660,13 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>2838081.612903226</v>
+        <v>-48347003.75</v>
       </c>
       <c r="E156" t="n">
-        <v>2488601.935483871</v>
+        <v>-52474763.75</v>
       </c>
       <c r="F156" t="n">
-        <v>2838081.612903226</v>
+        <v>-46220203.75</v>
       </c>
       <c r="G156" t="inlineStr">
         <is>
@@ -6499,7 +6679,7 @@
         </is>
       </c>
       <c r="I156" t="n">
-        <v>12.31394036839743</v>
+        <v>11.91917705394148</v>
       </c>
     </row>
     <row r="157">
@@ -6509,13 +6689,13 @@
         </is>
       </c>
       <c r="D157" t="n">
-        <v>22279561.62896263</v>
+        <v>273905077.3980494</v>
       </c>
       <c r="E157" t="n">
-        <v>19622065.81315529</v>
+        <v>273341695.35326</v>
       </c>
       <c r="F157" t="n">
-        <v>23884897.59634926</v>
+        <v>273905077.3980494</v>
       </c>
       <c r="G157" t="inlineStr">
         <is>
@@ -6524,11 +6704,11 @@
       </c>
       <c r="H157" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I157" t="n">
-        <v>17.84739401120788</v>
+        <v>0.2056851410500091</v>
       </c>
     </row>
     <row r="158">
@@ -6538,13 +6718,13 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>24504239.10251102</v>
+        <v>222928329.509829</v>
       </c>
       <c r="E158" t="n">
-        <v>21550431.56860603</v>
+        <v>218146838.3041205</v>
       </c>
       <c r="F158" t="n">
-        <v>26109575.06989764</v>
+        <v>225090763.6757569</v>
       </c>
       <c r="G158" t="inlineStr">
         <is>
@@ -6557,7 +6737,7 @@
         </is>
       </c>
       <c r="I158" t="n">
-        <v>17.46157679351877</v>
+        <v>3.084944605563252</v>
       </c>
     </row>
     <row r="159">
@@ -6567,13 +6747,13 @@
         </is>
       </c>
       <c r="D159" t="n">
-        <v>24504239.10251102</v>
+        <v>222928329.509829</v>
       </c>
       <c r="E159" t="n">
-        <v>21550431.56860603</v>
+        <v>218146838.3041205</v>
       </c>
       <c r="F159" t="n">
-        <v>26109575.06989764</v>
+        <v>225090763.6757569</v>
       </c>
       <c r="G159" t="inlineStr">
         <is>
@@ -6586,7 +6766,7 @@
         </is>
       </c>
       <c r="I159" t="n">
-        <v>17.46157679351876</v>
+        <v>3.084944605563252</v>
       </c>
     </row>
     <row r="160">
@@ -6596,13 +6776,13 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>120</v>
+        <v>5198</v>
       </c>
       <c r="E160" t="n">
-        <v>120</v>
+        <v>5192</v>
       </c>
       <c r="F160" t="n">
-        <v>122</v>
+        <v>5207</v>
       </c>
       <c r="G160" t="inlineStr">
         <is>
@@ -6615,7 +6795,7 @@
         </is>
       </c>
       <c r="I160" t="n">
-        <v>1.639344262295082</v>
+        <v>0.2880737468792011</v>
       </c>
     </row>
     <row r="161">
@@ -6625,26 +6805,26 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>1307849.99746176</v>
+        <v>1168693.745040697</v>
       </c>
       <c r="E161" t="n">
-        <v>1307834.795906328</v>
+        <v>1168596.610239464</v>
       </c>
       <c r="F161" t="n">
-        <v>1307862.86715619</v>
+        <v>1168799.358557804</v>
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>첨예형</t>
+          <t>평탄형</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>첨예형</t>
         </is>
       </c>
       <c r="I161" t="n">
-        <v>0.002146345046327881</v>
+        <v>0.01734671711232556</v>
       </c>
     </row>
     <row r="162">
@@ -6678,13 +6858,13 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>2838081.612903226</v>
+        <v>-43825083.75</v>
       </c>
       <c r="E163" t="n">
-        <v>2488601.935483871</v>
+        <v>-50617843.75</v>
       </c>
       <c r="F163" t="n">
-        <v>2838081.612903226</v>
+        <v>-39506483.75</v>
       </c>
       <c r="G163" t="inlineStr">
         <is>
@@ -6697,7 +6877,7 @@
         </is>
       </c>
       <c r="I163" t="n">
-        <v>12.31394036839743</v>
+        <v>21.95146844831769</v>
       </c>
     </row>
     <row r="164">
@@ -6707,13 +6887,13 @@
         </is>
       </c>
       <c r="D164" t="n">
-        <v>23272029.67227682</v>
+        <v>425243755.2360973</v>
       </c>
       <c r="E164" t="n">
-        <v>20452277.86005339</v>
+        <v>424105698.3038983</v>
       </c>
       <c r="F164" t="n">
-        <v>24555709.08009543</v>
+        <v>425243755.2360973</v>
       </c>
       <c r="G164" t="inlineStr">
         <is>
@@ -6722,11 +6902,11 @@
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>기준</t>
         </is>
       </c>
       <c r="I164" t="n">
-        <v>16.71070139598712</v>
+        <v>0.2676246078127936</v>
       </c>
     </row>
     <row r="165">
@@ -6736,13 +6916,13 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>25496707.14582521</v>
+        <v>376575863.6532693</v>
       </c>
       <c r="E165" t="n">
-        <v>22331217.54167268</v>
+        <v>368453344.4862061</v>
       </c>
       <c r="F165" t="n">
-        <v>26780386.55364382</v>
+        <v>380996268.6021094</v>
       </c>
       <c r="G165" t="inlineStr">
         <is>
@@ -6755,7 +6935,7 @@
         </is>
       </c>
       <c r="I165" t="n">
-        <v>16.61353544340745</v>
+        <v>3.292138309365567</v>
       </c>
     </row>
     <row r="166">
@@ -6765,13 +6945,13 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>25496707.14582521</v>
+        <v>376575863.6532693</v>
       </c>
       <c r="E166" t="n">
-        <v>22331217.54167268</v>
+        <v>368453344.4862061</v>
       </c>
       <c r="F166" t="n">
-        <v>26780386.55364381</v>
+        <v>380996268.6021094</v>
       </c>
       <c r="G166" t="inlineStr">
         <is>
@@ -6784,7 +6964,7 @@
         </is>
       </c>
       <c r="I166" t="n">
-        <v>16.61353544340744</v>
+        <v>3.292138309365567</v>
       </c>
     </row>
     <row r="167">
@@ -6794,13 +6974,13 @@
         </is>
       </c>
       <c r="D167" t="n">
-        <v>120</v>
+        <v>5186</v>
       </c>
       <c r="E167" t="n">
-        <v>120</v>
+        <v>5175</v>
       </c>
       <c r="F167" t="n">
-        <v>122</v>
+        <v>5204</v>
       </c>
       <c r="G167" t="inlineStr">
         <is>
@@ -6813,7 +6993,7 @@
         </is>
       </c>
       <c r="I167" t="n">
-        <v>1.639344262295082</v>
+        <v>0.5572636433512683</v>
       </c>
     </row>
     <row r="168">
@@ -6823,26 +7003,26 @@
         </is>
       </c>
       <c r="D168" t="n">
-        <v>2615699.994923521</v>
+        <v>2337387.490081393</v>
       </c>
       <c r="E168" t="n">
-        <v>2615669.591812657</v>
+        <v>2337193.220478929</v>
       </c>
       <c r="F168" t="n">
-        <v>2615725.734312381</v>
+        <v>2337598.717115608</v>
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>첨예형</t>
+          <t>평탄형</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>평탄형</t>
+          <t>첨예형</t>
         </is>
       </c>
       <c r="I168" t="n">
-        <v>0.002146345046327881</v>
+        <v>0.01734671711232556</v>
       </c>
     </row>
     <row r="169">
@@ -6866,8 +7046,607 @@
       </c>
       <c r="I169" t="inlineStr"/>
     </row>
+    <row r="170">
+      <c r="A170" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B170" t="n">
+        <v>500</v>
+      </c>
+      <c r="C170" t="inlineStr">
+        <is>
+          <t>기본요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D170" t="n">
+        <v>1371755.161290321</v>
+      </c>
+      <c r="E170" t="n">
+        <v>1019989.032258064</v>
+      </c>
+      <c r="F170" t="n">
+        <v>1421135.161290321</v>
+      </c>
+      <c r="G170" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H170" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I170" t="n">
+        <v>28.22716233887541</v>
+      </c>
+    </row>
+    <row r="171">
+      <c r="C171" t="inlineStr">
+        <is>
+          <t>전력량요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>21832794.0374309</v>
+      </c>
+      <c r="E171" t="n">
+        <v>19707849.27224809</v>
+      </c>
+      <c r="F171" t="n">
+        <v>23383003.92461409</v>
+      </c>
+      <c r="G171" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H171" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I171" t="n">
+        <v>15.71720495884344</v>
+      </c>
+    </row>
+    <row r="172">
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>절감액(원)</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>22552939.7162026</v>
+      </c>
+      <c r="E172" t="n">
+        <v>20181372.38521974</v>
+      </c>
+      <c r="F172" t="n">
+        <v>24100050.37364634</v>
+      </c>
+      <c r="G172" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H172" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I172" t="n">
+        <v>16.26004065415448</v>
+      </c>
+    </row>
+    <row r="173">
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>12개월 환산 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>22552939.7162026</v>
+      </c>
+      <c r="E173" t="n">
+        <v>20181372.38521974</v>
+      </c>
+      <c r="F173" t="n">
+        <v>24100050.37364634</v>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H173" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I173" t="n">
+        <v>16.26004065415447</v>
+      </c>
+    </row>
+    <row r="174">
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>요금적용전력(kW)</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>120</v>
+      </c>
+      <c r="E174" t="n">
+        <v>120</v>
+      </c>
+      <c r="F174" t="n">
+        <v>122</v>
+      </c>
+      <c r="G174" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="H174" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="I174" t="n">
+        <v>1.639344262295082</v>
+      </c>
+    </row>
+    <row r="175">
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>발전량(kWh)</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>653924.9987308802</v>
+      </c>
+      <c r="E175" t="n">
+        <v>653917.3979531642</v>
+      </c>
+      <c r="F175" t="n">
+        <v>653931.4335780952</v>
+      </c>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H175" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I175" t="n">
+        <v>0.002146345046327881</v>
+      </c>
+    </row>
+    <row r="176">
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>회수기간(년)</t>
+        </is>
+      </c>
+      <c r="D176" t="inlineStr"/>
+      <c r="E176" t="inlineStr"/>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H176" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr"/>
+    </row>
+    <row r="177">
+      <c r="B177" t="n">
+        <v>1000</v>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>기본요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="E177" t="n">
+        <v>2488601.935483871</v>
+      </c>
+      <c r="F177" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H177" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I177" t="n">
+        <v>12.31394036839743</v>
+      </c>
+    </row>
+    <row r="178">
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>전력량요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>22279561.62896263</v>
+      </c>
+      <c r="E178" t="n">
+        <v>19622065.81315529</v>
+      </c>
+      <c r="F178" t="n">
+        <v>23884897.59634926</v>
+      </c>
+      <c r="G178" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H178" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I178" t="n">
+        <v>17.84739401120788</v>
+      </c>
+    </row>
+    <row r="179">
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>절감액(원)</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>24504239.10251102</v>
+      </c>
+      <c r="E179" t="n">
+        <v>21550431.56860603</v>
+      </c>
+      <c r="F179" t="n">
+        <v>26109575.06989764</v>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H179" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I179" t="n">
+        <v>17.46157679351877</v>
+      </c>
+    </row>
+    <row r="180">
+      <c r="C180" t="inlineStr">
+        <is>
+          <t>12개월 환산 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D180" t="n">
+        <v>24504239.10251102</v>
+      </c>
+      <c r="E180" t="n">
+        <v>21550431.56860603</v>
+      </c>
+      <c r="F180" t="n">
+        <v>26109575.06989764</v>
+      </c>
+      <c r="G180" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H180" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I180" t="n">
+        <v>17.46157679351876</v>
+      </c>
+    </row>
+    <row r="181">
+      <c r="C181" t="inlineStr">
+        <is>
+          <t>요금적용전력(kW)</t>
+        </is>
+      </c>
+      <c r="D181" t="n">
+        <v>120</v>
+      </c>
+      <c r="E181" t="n">
+        <v>120</v>
+      </c>
+      <c r="F181" t="n">
+        <v>122</v>
+      </c>
+      <c r="G181" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="H181" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="I181" t="n">
+        <v>1.639344262295082</v>
+      </c>
+    </row>
+    <row r="182">
+      <c r="C182" t="inlineStr">
+        <is>
+          <t>발전량(kWh)</t>
+        </is>
+      </c>
+      <c r="D182" t="n">
+        <v>1307849.99746176</v>
+      </c>
+      <c r="E182" t="n">
+        <v>1307834.795906328</v>
+      </c>
+      <c r="F182" t="n">
+        <v>1307862.86715619</v>
+      </c>
+      <c r="G182" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H182" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I182" t="n">
+        <v>0.002146345046327881</v>
+      </c>
+    </row>
+    <row r="183">
+      <c r="C183" t="inlineStr">
+        <is>
+          <t>회수기간(년)</t>
+        </is>
+      </c>
+      <c r="D183" t="inlineStr"/>
+      <c r="E183" t="inlineStr"/>
+      <c r="F183" t="inlineStr"/>
+      <c r="G183" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H183" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I183" t="inlineStr"/>
+    </row>
+    <row r="184">
+      <c r="B184" t="n">
+        <v>2000</v>
+      </c>
+      <c r="C184" t="inlineStr">
+        <is>
+          <t>기본요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D184" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="E184" t="n">
+        <v>2488601.935483871</v>
+      </c>
+      <c r="F184" t="n">
+        <v>2838081.612903226</v>
+      </c>
+      <c r="G184" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H184" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I184" t="n">
+        <v>12.31394036839743</v>
+      </c>
+    </row>
+    <row r="185">
+      <c r="C185" t="inlineStr">
+        <is>
+          <t>전력량요금 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D185" t="n">
+        <v>23272029.67227682</v>
+      </c>
+      <c r="E185" t="n">
+        <v>20452277.86005339</v>
+      </c>
+      <c r="F185" t="n">
+        <v>24555709.08009543</v>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H185" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I185" t="n">
+        <v>16.71070139598712</v>
+      </c>
+    </row>
+    <row r="186">
+      <c r="C186" t="inlineStr">
+        <is>
+          <t>절감액(원)</t>
+        </is>
+      </c>
+      <c r="D186" t="n">
+        <v>25496707.14582521</v>
+      </c>
+      <c r="E186" t="n">
+        <v>22331217.54167268</v>
+      </c>
+      <c r="F186" t="n">
+        <v>26780386.55364382</v>
+      </c>
+      <c r="G186" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H186" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I186" t="n">
+        <v>16.61353544340745</v>
+      </c>
+    </row>
+    <row r="187">
+      <c r="C187" t="inlineStr">
+        <is>
+          <t>12개월 환산 절감액(원)</t>
+        </is>
+      </c>
+      <c r="D187" t="n">
+        <v>25496707.14582521</v>
+      </c>
+      <c r="E187" t="n">
+        <v>22331217.54167268</v>
+      </c>
+      <c r="F187" t="n">
+        <v>26780386.55364381</v>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H187" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I187" t="n">
+        <v>16.61353544340744</v>
+      </c>
+    </row>
+    <row r="188">
+      <c r="C188" t="inlineStr">
+        <is>
+          <t>요금적용전력(kW)</t>
+        </is>
+      </c>
+      <c r="D188" t="n">
+        <v>120</v>
+      </c>
+      <c r="E188" t="n">
+        <v>120</v>
+      </c>
+      <c r="F188" t="n">
+        <v>122</v>
+      </c>
+      <c r="G188" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="H188" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="I188" t="n">
+        <v>1.639344262295082</v>
+      </c>
+    </row>
+    <row r="189">
+      <c r="C189" t="inlineStr">
+        <is>
+          <t>발전량(kWh)</t>
+        </is>
+      </c>
+      <c r="D189" t="n">
+        <v>2615699.994923521</v>
+      </c>
+      <c r="E189" t="n">
+        <v>2615669.591812657</v>
+      </c>
+      <c r="F189" t="n">
+        <v>2615725.734312381</v>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>첨예형</t>
+        </is>
+      </c>
+      <c r="H189" t="inlineStr">
+        <is>
+          <t>평탄형</t>
+        </is>
+      </c>
+      <c r="I189" t="n">
+        <v>0.002146345046327881</v>
+      </c>
+    </row>
+    <row r="190">
+      <c r="C190" t="inlineStr">
+        <is>
+          <t>회수기간(년)</t>
+        </is>
+      </c>
+      <c r="D190" t="inlineStr"/>
+      <c r="E190" t="inlineStr"/>
+      <c r="F190" t="inlineStr"/>
+      <c r="G190" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="H190" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I190" t="inlineStr"/>
+    </row>
   </sheetData>
-  <mergeCells count="32">
+  <mergeCells count="36">
     <mergeCell ref="A44:A64"/>
     <mergeCell ref="B86:B92"/>
     <mergeCell ref="B44:B50"/>
@@ -6876,8 +7655,10 @@
     <mergeCell ref="A23:A43"/>
     <mergeCell ref="B107:B113"/>
     <mergeCell ref="B37:B43"/>
+    <mergeCell ref="B177:B183"/>
     <mergeCell ref="B128:B134"/>
     <mergeCell ref="B65:B71"/>
+    <mergeCell ref="A170:A190"/>
     <mergeCell ref="A107:A127"/>
     <mergeCell ref="B142:B148"/>
     <mergeCell ref="A128:A148"/>
@@ -6890,12 +7671,14 @@
     <mergeCell ref="B135:B141"/>
     <mergeCell ref="A65:A85"/>
     <mergeCell ref="A149:A169"/>
+    <mergeCell ref="B184:B190"/>
     <mergeCell ref="A86:A106"/>
     <mergeCell ref="B72:B78"/>
     <mergeCell ref="A2:A22"/>
     <mergeCell ref="B100:B106"/>
     <mergeCell ref="B149:B155"/>
     <mergeCell ref="B156:B162"/>
+    <mergeCell ref="B170:B176"/>
     <mergeCell ref="B121:B127"/>
     <mergeCell ref="B2:B8"/>
     <mergeCell ref="B93:B99"/>
@@ -6911,7 +7694,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -7315,7 +8098,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C8 역률 미달형</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -7324,13 +8107,13 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>62942872.33519353</v>
+        <v>3357428545.0455</v>
       </c>
       <c r="D23" t="n">
-        <v>-922938.8148709536</v>
+        <v>0</v>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="24">
@@ -7340,13 +8123,13 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>62019933.52032258</v>
+        <v>3304814805.048</v>
       </c>
       <c r="D24" t="n">
-        <v>0</v>
+        <v>52613739.99750042</v>
       </c>
       <c r="E24" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="25">
@@ -7356,40 +8139,94 @@
         </is>
       </c>
       <c r="C25" t="n">
+        <v>3333774505.65975</v>
+      </c>
+      <c r="D25" t="n">
+        <v>23654039.38575029</v>
+      </c>
+      <c r="E25" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>I</t>
+        </is>
+      </c>
+      <c r="C26" t="n">
+        <v>62942872.33519353</v>
+      </c>
+      <c r="D26" t="n">
+        <v>-922938.8148709536</v>
+      </c>
+      <c r="E26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>II</t>
+        </is>
+      </c>
+      <c r="C27" t="n">
+        <v>62019933.52032258</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>III</t>
+        </is>
+      </c>
+      <c r="C28" t="n">
         <v>68875492.43619356</v>
       </c>
-      <c r="D25" t="n">
+      <c r="D28" t="n">
         <v>-6855558.915870979</v>
       </c>
-      <c r="E25" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" t="inlineStr">
+      <c r="E28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" t="inlineStr">
         <is>
           <t>IV</t>
         </is>
       </c>
-      <c r="C26" t="n">
+      <c r="C29" t="n">
         <v>68298776.96832258</v>
       </c>
-      <c r="D26" t="n">
+      <c r="D29" t="n">
         <v>-6278843.447999999</v>
       </c>
-      <c r="E26" t="b">
+      <c r="E29" t="b">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A8:A10"/>
-    <mergeCell ref="A23:A26"/>
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A17:A19"/>
+    <mergeCell ref="A26:A29"/>
     <mergeCell ref="A20:A22"/>
     <mergeCell ref="A11:A13"/>
     <mergeCell ref="A5:A7"/>
+    <mergeCell ref="A23:A25"/>
     <mergeCell ref="A14:A16"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -7402,7 +8239,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F41"/>
+  <dimension ref="A1:F46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8220,7 +9057,7 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C8 역률 미달형</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
@@ -8229,10 +9066,10 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>0</v>
+        <v>52613739.99750042</v>
       </c>
       <c r="D37" t="n">
-        <v>0</v>
+        <v>52613739.99750042</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -8241,7 +9078,7 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>II → II</t>
+          <t>I → II</t>
         </is>
       </c>
     </row>
@@ -8262,7 +9099,7 @@
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>계약 290 kW (실제 값)</t>
+          <t>계약 5,823 kW 가정 (관측 최대 × 1.1)</t>
         </is>
       </c>
     </row>
@@ -8273,10 +9110,10 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>124225.2129032239</v>
+        <v>4528045.5625</v>
       </c>
       <c r="D39" t="n">
-        <v>124225.2129032239</v>
+        <v>4528045.5625</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -8295,7 +9132,9 @@
           <t>7.6 ESS</t>
         </is>
       </c>
-      <c r="C40" t="inlineStr"/>
+      <c r="C40" t="n">
+        <v>8349096.652772427</v>
+      </c>
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
@@ -8304,7 +9143,7 @@
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>최소 규격 미달 — 필요 출력 25.3 kW &lt; 상업용 최소 50 kW</t>
+          <t>목표 5,180 kW (기준 5,293.0 → 실제 5,180.0) · 150 kW / 100 kWh · 회수 31.4년</t>
         </is>
       </c>
     </row>
@@ -8323,17 +9162,128 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
+          <t>거래 가능일 245일 · 등록 권장 2,011 kW · 연간 감축 34,350 kWh</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>R1 용인 실측</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>7.1 선택요금 전환</t>
+        </is>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>II → II</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>7.2 계약전력 조정</t>
+        </is>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="inlineStr"/>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>계약 290 kW (실제 값)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>7.4 역률 개선 (92→97%)</t>
+        </is>
+      </c>
+      <c r="C44" t="n">
+        <v>124225.2129032239</v>
+      </c>
+      <c r="D44" t="n">
+        <v>124225.2129032239</v>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>높음</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>요금표와 약관만으로 확정</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>7.6 ESS</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr"/>
+      <c r="D45" t="inlineStr"/>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>중간~낮음</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>최소 규격 미달 — 필요 출력 25.3 kW &lt; 상업용 최소 50 kW</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>7.3 경제성DR</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr"/>
+      <c r="D46" t="inlineStr"/>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>중간</t>
+        </is>
+      </c>
+      <c r="F46" t="inlineStr">
+        <is>
           <t>거래 가능일 244일 · 등록 권장 28 kW · 연간 감축 5,882 kWh</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
+  <mergeCells count="9">
     <mergeCell ref="A22:A26"/>
     <mergeCell ref="A17:A21"/>
     <mergeCell ref="A12:A16"/>
     <mergeCell ref="A27:A31"/>
     <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A42:A46"/>
     <mergeCell ref="A7:A11"/>
     <mergeCell ref="A37:A41"/>
     <mergeCell ref="A32:A36"/>
@@ -8348,7 +9298,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D119"/>
+  <dimension ref="A1:D133"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10077,7 +11027,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>R1 용인 실측</t>
+          <t>C8 역률 미달형</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -10109,7 +11059,7 @@
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>0 → 21,832,794 → 23,715,557 → 24,660,959</t>
+          <t>0 → 78,883,247 → 157,766,493 → 315,532,987</t>
         </is>
       </c>
     </row>
@@ -10126,7 +11076,7 @@
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>증분 1,371,755 → 49,380 → 0</t>
+          <t>증분 12,693,662 → 5,217,352 → 3,924,070</t>
         </is>
       </c>
     </row>
@@ -10143,7 +11093,7 @@
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>132.0 → 120.0 → 120.0 → 120.0</t>
+          <t>5,293.0 → 5,204.0 → 5,198.0 → 5,186.0</t>
         </is>
       </c>
     </row>
@@ -10160,7 +11110,7 @@
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>최대 편차 0.002%</t>
+          <t>최대 편차 0.017%</t>
         </is>
       </c>
     </row>
@@ -10194,7 +11144,7 @@
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>기본요금 절감액 상한: 평탄형</t>
+          <t>기본요금 절감액 상한: 기준, 평탄형</t>
         </is>
       </c>
     </row>
@@ -10211,7 +11161,7 @@
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>0 원 · II → II</t>
+          <t>52,613,740 원 · I → II</t>
         </is>
       </c>
     </row>
@@ -10228,7 +11178,7 @@
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>124,225 원 (기본요금 12,422,521 의 1.00%)</t>
+          <t>4,528,046 원 (기본요금 452,804,556 의 1.00%)</t>
         </is>
       </c>
     </row>
@@ -10245,7 +11195,7 @@
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>244 / 365일</t>
+          <t>245 / 359일</t>
         </is>
       </c>
     </row>
@@ -10262,7 +11212,7 @@
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>viable=False · 목표 0 kW</t>
+          <t>viable=True · 목표 5,180 kW</t>
         </is>
       </c>
     </row>
@@ -10279,7 +11229,7 @@
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>목표 0 kW · 절감액 —</t>
+          <t>목표 5,180 kW · 절감액 8,349,097 원</t>
         </is>
       </c>
     </row>
@@ -10296,7 +11246,7 @@
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>어긋난 점 0개 / 0개</t>
+          <t>어긋난 점 0개 / 21개</t>
         </is>
       </c>
     </row>
@@ -10313,19 +11263,19 @@
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>어긋난 점 0개 / 0개</t>
+          <t>어긋난 점 0개 / 21개</t>
         </is>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>교차</t>
+          <t>R1 용인 실측</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>C1 오전 피크형 &gt; C2 오후 피크형 (요금적용전력 저감 폭)</t>
+          <t>PV 0 kWp 절감액이 정확히 0</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -10335,14 +11285,14 @@
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>C1 95.0 kW vs C2 5.0 kW — C2 는 피크가 늦어 PV 가 깎은 뒤 저녁 슬롯이 새 최대가 된다</t>
+          <t>0.000000 원</t>
         </is>
       </c>
     </row>
     <row r="115">
       <c r="B115" t="inlineStr">
         <is>
-          <t>C3 평탄형은 기본요금 절감이 거의 없다 (절감의 대부분이 전력량요금)</t>
+          <t>용량 증가 시 전력량요금 절감액 단조 증가</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -10352,14 +11302,14 @@
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>기본요금 비중 C3 3.6% vs C1 10.2% (C3 저감 26.0 kW)</t>
+          <t>0 → 21,832,794 → 23,715,557 → 24,660,959</t>
         </is>
       </c>
     </row>
     <row r="116">
       <c r="B116" t="inlineStr">
         <is>
-          <t>C5 겨울 피크형은 기본요금 절감이 매우 작다</t>
+          <t>기본요금 절감액 단조 증가 후 포화</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -10369,14 +11319,14 @@
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>저감률 C5 0.29% vs C1 1.79% — 겨울 대상월의 피크가 07~09시·17~20시라 PV 가 닿지 않는다</t>
+          <t>증분 1,371,755 → 49,380 → 0</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="B117" t="inlineStr">
         <is>
-          <t>C6 야간 피크형: 요금적용전력 &lt; 관측 최대수요 (경부하 제외, 5.2 ①)</t>
+          <t>용량 증가 시 요금적용전력 단조 감소</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -10386,14 +11336,14 @@
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>관측 10,920.6 kW vs 요금적용 3,604.0 kW (67.0% 낮다)</t>
+          <t>132.0 → 120.0 → 120.0 → 120.0</t>
         </is>
       </c>
     </row>
     <row r="118">
       <c r="B118" t="inlineStr">
         <is>
-          <t>C6 야간 피크형: 하한이 요금적용전력을 붙들어 PV 가 한 칸도 못 내린다</t>
+          <t>감도 세 시나리오의 발전량이 ±1% 이내 (총량 보존)</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
@@ -10403,38 +11353,282 @@
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>C6 저감 0.00 kW vs C1 95.00 kW — 경부하 최대라 대상 수요가 하한 3,603.8 kW 아래에 있다</t>
+          <t>최대 편차 0.002%</t>
         </is>
       </c>
     </row>
     <row r="119">
       <c r="B119" t="inlineStr">
         <is>
+          <t>기준값이 범위 안에 있음</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>벗어난 지표 0건</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>상한 시나리오 기록 (단조성은 요구하지 않는다)</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>기본요금 절감액 상한: 평탄형</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>선택요금 전환 절감액 ≥ 0 (확정 계산)</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>0 원 · II → II</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>역률 개선 절감액 = 기본요금의 1.0% (감액 상한)</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>124,225 원 (기본요금 12,422,521 의 1.00%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>DR 거래 가능일이 전체 일수보다 적음 (토·일·공휴일 제외)</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>244 / 365일</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>ESS 성립하지 않으면 목표가 0 (없는 목표를 내지 않는다)</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>viable=False · 목표 0 kW</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>ESS 목표를 냈으면 절감액 &gt; 0</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>목표 0 kW · 절감액 —</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>ESS 목표 달성이면 실제 요금적용전력이 목표 이하</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>어긋난 점 0개 / 0개</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>ESS 절감액이 0 이하인 점에는 회수기간이 없다</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>어긋난 점 0개 / 0개</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>교차</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>C1 오전 피크형 &gt; C2 오후 피크형 (요금적용전력 저감 폭)</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>C1 95.0 kW vs C2 5.0 kW — C2 는 피크가 늦어 PV 가 깎은 뒤 저녁 슬롯이 새 최대가 된다</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>C3 평탄형은 기본요금 절감이 거의 없다 (절감의 대부분이 전력량요금)</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>기본요금 비중 C3 3.6% vs C1 10.2% (C3 저감 26.0 kW)</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>C5 겨울 피크형은 기본요금 절감이 매우 작다</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>저감률 C5 0.29% vs C1 1.79% — 겨울 대상월의 피크가 07~09시·17~20시라 PV 가 닿지 않는다</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>C6 야간 피크형: 요금적용전력 &lt; 관측 최대수요 (경부하 제외, 5.2 ①)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>관측 10,920.6 kW vs 요금적용 3,604.0 kW (67.0% 낮다)</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>C6 야간 피크형: 하한이 요금적용전력을 붙들어 PV 가 한 칸도 못 내린다</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>C6 저감 0.00 kW vs C1 95.00 kW — 경부하 최대라 대상 수요가 하한 3,603.8 kW 아래에 있다</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="B133" t="inlineStr">
+        <is>
           <t>C4 산업용(을) 주말 할인이 PV 최성기와 겹쳐 전력량요금 절감 비율이 낮다</t>
         </is>
       </c>
-      <c r="C119" t="inlineStr">
-        <is>
-          <t>통과</t>
-        </is>
-      </c>
-      <c r="D119" t="inlineStr">
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>통과</t>
+        </is>
+      </c>
+      <c r="D133" t="inlineStr">
         <is>
           <t>C4 4.95% vs C1 5.44% (봄·가을 토·일·공휴일 11~14시 할인 구간의 단가가 이미 낮다)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="9">
+  <mergeCells count="10">
     <mergeCell ref="A30:A43"/>
     <mergeCell ref="A44:A57"/>
     <mergeCell ref="A16:A29"/>
-    <mergeCell ref="A114:A119"/>
+    <mergeCell ref="A114:A127"/>
     <mergeCell ref="A100:A113"/>
     <mergeCell ref="A72:A85"/>
     <mergeCell ref="A86:A99"/>
     <mergeCell ref="A2:A15"/>
     <mergeCell ref="A58:A71"/>
+    <mergeCell ref="A128:A133"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -10446,7 +11640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -10469,7 +11663,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9.7 초</t>
+          <t>10.3 초</t>
         </is>
       </c>
     </row>
@@ -10481,7 +11675,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>9.8 초</t>
+          <t>10.4 초</t>
         </is>
       </c>
     </row>
@@ -10493,7 +11687,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>6.6 초</t>
+          <t>7.4 초</t>
         </is>
       </c>
     </row>
@@ -10505,7 +11699,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10.1 초</t>
+          <t>11.3 초</t>
         </is>
       </c>
     </row>
@@ -10517,7 +11711,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10.9 초</t>
+          <t>11.8 초</t>
         </is>
       </c>
     </row>
@@ -10529,7 +11723,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>8.5 초</t>
+          <t>9.1 초</t>
         </is>
       </c>
     </row>
@@ -10541,55 +11735,67 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10.1 초</t>
+          <t>10.6 초</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>R1 용인 실측 소요</t>
+          <t>C8 역률 미달형 소요</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>15.2 초</t>
+          <t>12.7 초</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>전체 소요</t>
+          <t>R1 용인 실측 소요</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>84.3 초</t>
+          <t>16.2 초</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>기상 취득 호출</t>
+          <t>전체 소요</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>0 회</t>
+          <t>103.6 초</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>기상 취득 호출</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>0 회</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>기상 캐시 적중</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>8/8 (C1~C7 은 좌표·기간이 같아 첫 건만 취득한다. 실측은 따로 선다)</t>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>9/9 (C1~C8 은 좌표·기간이 같아 첫 건만 취득한다. 실측은 따로 선다)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S143 5절: 마감 - 1,691건 3분 39초 · 케이스 132/132 · 감사 넷 불변 (미해결 67 -> 66)
pytest **1,691 passed · xfailed 0 · failed 0 · skip 0**(수집 1,691 · 1번 PC ·
앞단 전체 · 일꾼 8 · 깨끗한 판) · 케이스 **132/132 · 회귀값 여덟 불변 ·
기상 취득 0회 · 124.7초** · 화면 감사 **957·807·961·808 불변** ·
`scan_ctrl` 0곳 · `ruff check` 통과 · `ruff format` 어긋남 **여덟**(불변) ·
`mypy` **110파일 무결** · 살아 있는 못 **0건**.

건수가 1,688 → 1,691 로 셋 늘었다 — 이 판이 세운 못 셋이다.

미해결 **67 → 66**. 줄어든 것 넷 — PPT 와 Word 가 부가금을 「안 쟀다」 고
말하지 않는다 · 계약전력 조정이 300 kW 종별 경계를 안 본다 · 초과가 나는
벌에서 계약전력 조정이 목표도 부가금 금액도 안 낸다 · 종별 문턱 안내가
계약전력 기준 종별에서만 뜬다. 늘어난 것 셋 — 종별 문턱이 요금표와
rules_kr.json 두 자리에 있고 정본이 안 정해졌다 · 초과 벌의 상향 목표와
몫이 PPT·Excel 에 안 선다 · 미해결 갈래 훑기 결과가 보고에만 있고 저장소에
안 남는다.

**돌고 있는 백그라운드 셸 없음** — 모두 앞단에서 돌렸다. 마감 시점에 다른
프로젝트 python **0개**.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>10.97319450000214</v>
+        <v>12.57262709999486</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>11.78684829999838</v>
+        <v>12.38415569999779</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>7.000835599996208</v>
+        <v>8.185998100001598</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>11.4225632000016</v>
+        <v>14.26996710000094</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>13.18067620000511</v>
+        <v>14.92204119999951</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>9.968419899996661</v>
+        <v>11.45763729999453</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>13.52733950000402</v>
+        <v>13.22472720000223</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>12.5918210000018</v>
+        <v>14.88549209999474</v>
       </c>
     </row>
     <row r="10">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>17.77583449999656</v>
+        <v>18.27427670000179</v>
       </c>
     </row>
   </sheetData>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>11.0 초</t>
+          <t>12.6 초</t>
         </is>
       </c>
     </row>
@@ -11675,7 +11675,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>11.8 초</t>
+          <t>12.4 초</t>
         </is>
       </c>
     </row>
@@ -11687,7 +11687,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>7.0 초</t>
+          <t>8.2 초</t>
         </is>
       </c>
     </row>
@@ -11699,7 +11699,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>11.4 초</t>
+          <t>14.3 초</t>
         </is>
       </c>
     </row>
@@ -11711,7 +11711,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13.2 초</t>
+          <t>14.9 초</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10.0 초</t>
+          <t>11.5 초</t>
         </is>
       </c>
     </row>
@@ -11735,7 +11735,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.5 초</t>
+          <t>13.2 초</t>
         </is>
       </c>
     </row>
@@ -11747,7 +11747,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>12.6 초</t>
+          <t>14.9 초</t>
         </is>
       </c>
     </row>
@@ -11759,7 +11759,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>17.8 초</t>
+          <t>18.3 초</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>112.3 초</t>
+          <t>124.7 초</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
S144 4절: 마감 - 1,691건 3분 28초 · 케이스 132/132 · 감사 넷 불변 (미해결 66 -> 66)
앞단 전체 pytest 1,691 passed · xfailed 0 · failed 0 · skip 0 · 3분 28초
(깨끗한 판 · 앞뒤로 남의 python 0개). 건수가 앞 판과 같다 — 시험을 안 더했다.
케이스 132/132 · 회귀값 여덟 불변 · 기상 취득 0회 · 도구 95.9초.
화면 감사 957·807·961·808 불변 — src\ 를 안 고친 판이라 움직이면 결함이었다.
scan_ctrl 0곳 · ruff check 통과 · ruff format 어긋남 여덟(앞 판과 같다) ·
맨 mypy 10건 파일 둘 · mypy src 무결 110파일.

「mypy 범위」 칸을 실물로 고쳤다 — 167 -> 168파일. S141 이
tests\test_base_fee_definition.py 를 더한 몫이고, S135 이후 새 파이썬 파일이
그 하나뿐인 것을 git diff --name-status 로 봤다.

미해결 66 -> 66 (줄어든 것 하나 · 늘어난 것 하나 · 이름은 절에 있다).
세션 목록표에 144세션 행을 세웠다. 지시서를 docs\directives\S144.md 로 앉히고
인수인계를 docs\2026-09-07_인수인계.md 로 남겼다.

살아 있는 못 0건. 백그라운드 셸 없음. src\ 0줄.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XJ2ZbB4RPSZ6y6vQgneDjR
</commit_message>
<xml_diff>
--- a/output/casestudy_20260907.xlsx
+++ b/output/casestudy_20260907.xlsx
@@ -544,7 +544,7 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>12.57262709999486</v>
+        <v>11.1845100999999</v>
       </c>
     </row>
     <row r="3">
@@ -596,7 +596,7 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>12.38415569999779</v>
+        <v>10.47643500000413</v>
       </c>
     </row>
     <row r="4">
@@ -648,7 +648,7 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>8.185998100001598</v>
+        <v>6.308381199996802</v>
       </c>
     </row>
     <row r="5">
@@ -700,7 +700,7 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>14.26996710000094</v>
+        <v>9.850841800005583</v>
       </c>
     </row>
     <row r="6">
@@ -752,7 +752,7 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>14.92204119999951</v>
+        <v>10.86357459999999</v>
       </c>
     </row>
     <row r="7">
@@ -804,7 +804,7 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>11.45763729999453</v>
+        <v>8.465750700001081</v>
       </c>
     </row>
     <row r="8">
@@ -856,7 +856,7 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>13.22472720000223</v>
+        <v>10.36475020000216</v>
       </c>
     </row>
     <row r="9">
@@ -908,7 +908,7 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>14.88549209999474</v>
+        <v>10.82911839999724</v>
       </c>
     </row>
     <row r="10">
@@ -960,7 +960,7 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>18.27427670000179</v>
+        <v>14.12262300000293</v>
       </c>
     </row>
   </sheetData>
@@ -11663,7 +11663,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>12.6 초</t>
+          <t>11.2 초</t>
         </is>
       </c>
     </row>
@@ -11675,7 +11675,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>12.4 초</t>
+          <t>10.5 초</t>
         </is>
       </c>
     </row>
@@ -11687,7 +11687,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>8.2 초</t>
+          <t>6.3 초</t>
         </is>
       </c>
     </row>
@@ -11699,7 +11699,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>14.3 초</t>
+          <t>9.9 초</t>
         </is>
       </c>
     </row>
@@ -11711,7 +11711,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>14.9 초</t>
+          <t>10.9 초</t>
         </is>
       </c>
     </row>
@@ -11723,7 +11723,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>11.5 초</t>
+          <t>8.5 초</t>
         </is>
       </c>
     </row>
@@ -11735,7 +11735,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13.2 초</t>
+          <t>10.4 초</t>
         </is>
       </c>
     </row>
@@ -11747,7 +11747,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>14.9 초</t>
+          <t>10.8 초</t>
         </is>
       </c>
     </row>
@@ -11759,7 +11759,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>18.3 초</t>
+          <t>14.1 초</t>
         </is>
       </c>
     </row>
@@ -11771,7 +11771,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>124.7 초</t>
+          <t>95.9 초</t>
         </is>
       </c>
     </row>

</xml_diff>